<commit_message>
Social v2 without people (produce cut-outs + bold type, 60 posts) and forest-green packaging with 12 new mockups
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/Fresh-Valley-Social-Calendar.xlsx
+++ b/files/Fresh-Valley-Social-Calendar.xlsx
@@ -327,7 +327,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lifestyle photo</t>
+          <t xml:space="preserve">Produce crowd + serif</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -337,12 +337,12 @@
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Picked this morning. At your table today.</t>
+          <t xml:space="preserve">Fresh feels different.</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">اتقطف الصبح — على سفرتك النهارده</t>
+          <t xml:space="preserve">الفريش إحساسه مختلف</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -352,7 +352,7 @@
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">اتقطف الصبح — على سفرتك النهارده. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">الفريش إحساسه مختلف. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -390,7 +390,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product on white</t>
+          <t xml:space="preserve">Giant word + produce</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -400,12 +400,12 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sun, bottled.</t>
+          <t xml:space="preserve">Sun, in a peel.</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">شمس في قشرة</t>
+          <t xml:space="preserve">برتقال — شمس في قشرة</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -415,7 +415,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">شمس في قشرة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">برتقال — شمس في قشرة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -453,7 +453,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type on forest</t>
+          <t xml:space="preserve">Type statement</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -516,7 +516,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split photo</t>
+          <t xml:space="preserve">Glass pill on green</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -526,22 +526,22 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">A bowl of oranges changes the room.</t>
+          <t xml:space="preserve">Smell it before you see it.</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">طبق برتقال بيغيّر المكان كله</t>
+          <t xml:space="preserve">نعناع فريش لصباح أهدى</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The first thing on the island every morning. Navel oranges, delivered the day they’re picked. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Mint cut the morning it ships. Still lively when it arrives. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">طبق برتقال بيغيّر المكان كله. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">نعناع فريش لصباح أهدى. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box feature</t>
+          <t xml:space="preserve">Packaging feature</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -589,22 +589,22 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bring a box, not a bag of sweets.</t>
+          <t xml:space="preserve">Six fruits at their peak.</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">هات بوكس، مش علبة حلويات</t>
+          <t xml:space="preserve">البستان — ٦ فواكه في عزّها</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Host box arrives as a serving tray: grapes in the middle, dates, figs, strawberries and mint around it. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The Orchard box: mango, grapes, figs, pomegranates, oranges and peaches — each in its own well. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">هات بوكس، مش علبة حلويات. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">البستان — ٦ فواكه في عزّها. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product on white</t>
+          <t xml:space="preserve">Scattered letters</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -652,22 +652,22 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Red, ripe, and ready.</t>
+          <t xml:space="preserve">Soft, sweet, and whole.</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">حمرا ومستوية وجاهزة</t>
+          <t xml:space="preserve">تين بنفسجي من مطروح</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Winter strawberries are back. Picked at full colour and chilled within hours. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Purple figs from Matrouh are here. Soft, sweet and delivered whole. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">حمرا ومستوية وجاهزة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">تين بنفسجي من مطروح. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Framed photo</t>
+          <t xml:space="preserve">Label strips</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inside our packing house in Obour: every orange and every bunch is checked by hand before it is packed. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Every pomegranate is checked by hand before it is packed. Not perfect? It does not go in your box. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
@@ -761,14 +761,14 @@
       <c r="C12" s="7">
         <v>46336</v>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Box</t>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Season</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pattern card</t>
+          <t xml:space="preserve">Four colour tiles</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -778,27 +778,27 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The box becomes a tray.</t>
+          <t xml:space="preserve">Four colours of winter.</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">البوكس يبقى صينية</t>
+          <t xml:space="preserve">أربع ألوان للشتا</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lift the base out by its handles and it goes straight to the table. Nothing goes in the bin. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Oranges, lemons, romaine and beetroot — this week’s colours, picked whole. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">البوكس يبقى صينية. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">أربع ألوان للشتا. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lifestyle photo</t>
+          <t xml:space="preserve">Split: type over produce</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -841,22 +841,22 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smell it before you see it.</t>
+          <t xml:space="preserve">Fresh by the valley.</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ريحته بتوصل قبله</t>
+          <t xml:space="preserve">من الوادي لسفرتك — طازة كل يوم</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mint cut the morning it ships. Still lively when it arrives. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Vegetables picked at dawn and on your counter before lunch. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ريحته بتوصل قبله. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">من الوادي لسفرتك — طازة كل يوم. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Host tip</t>
+          <t xml:space="preserve">Wordmark block</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -904,22 +904,22 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dates first. Always.</t>
+          <t xml:space="preserve">Bring a box, not a bag of sweets.</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">التمر الأول — دايمًا</t>
+          <t xml:space="preserve">هات بوكس، مش علبة حلويات</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The host’s first gesture: a small bowl of Medjool dates by the door, before anything else. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The host’s gesture: a box of whole fruit instead of sweets. It says more. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">التمر الأول — دايمًا. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">هات بوكس، مش علبة حلويات. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lifestyle photo</t>
+          <t xml:space="preserve">Giant word + produce</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -967,22 +967,22 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The table is the point.</t>
+          <t xml:space="preserve">The middle of every table.</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">السفرة هي الحكاية</t>
+          <t xml:space="preserve">عنب أحمر — نص السفرة</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Friday lunch in the garden. Everything on the table was picked this week. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Red grapes from Minya. The first thing guests reach for. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">السفرة هي الحكاية. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">عنب أحمر — نص السفرة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Angle grid</t>
+          <t xml:space="preserve">Four colour tiles</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1030,22 +1030,22 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pomegranates &amp; figs.</t>
+          <t xml:space="preserve">Autumn, whole.</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">رمان وتين — أهلاً بالخريف</t>
+          <t xml:space="preserve">الخريف — كامل</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pomegranates from Assiut and purple figs from Matrouh. Autumn, whole and spotless. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Pomegranates, figs, dates and persimmon. Autumn, whole and spotless. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">رمان وتين — أهلاً بالخريف. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">الخريف — كامل. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type on forest</t>
+          <t xml:space="preserve">Type statement</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box feature</t>
+          <t xml:space="preserve">Packaging feature</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1156,22 +1156,22 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Six wells. Six fruits at their peak.</t>
+          <t xml:space="preserve">The week, sorted.</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">٦ خانات و٦ فواكه في عزّها</t>
+          <t xml:space="preserve">السوق — الأسبوع كله متقسم</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Orchard box: mango, grapes, figs, pomegranates, oranges and peaches — each in its own well. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The Market box: fruit on one side, vegetables on the other. The week, sorted. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">٦ خانات و٦ فواكه في عزّها. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">السوق — الأسبوع كله متقسم. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split photo</t>
+          <t xml:space="preserve">Glass pill on green</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lifestyle photo</t>
+          <t xml:space="preserve">Scattered letters</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1391,14 +1391,14 @@
       <c r="C22" s="7">
         <v>46350</v>
       </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Box</t>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The A Standard</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Framed photo</t>
+          <t xml:space="preserve">Label strips</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1408,27 +1408,27 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The card grows basil.</t>
+          <t xml:space="preserve">Picked at dawn. At your door by evening.</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الكارت يطلع ريحان</t>
+          <t xml:space="preserve">اتقطف الفجر — عندك بالليل</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Our grade card is made of seed paper. Plant it, water it, and basil comes up in about two weeks. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">From the farm to your door on the same day. Less time travelling, more time fresh. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الكارت يطلع ريحان. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">اتقطف الفجر — عندك بالليل. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -1454,14 +1454,14 @@
       <c r="C23" s="7">
         <v>46351</v>
       </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The A Standard</t>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Living Well</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product on white</t>
+          <t xml:space="preserve">Produce crowd + serif</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1471,27 +1471,27 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The host’s first gesture.</t>
+          <t xml:space="preserve">Eat the whole rainbow.</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">أول حاجة بيقدّمها المُضيف</t>
+          <t xml:space="preserve">كُل قوس قزح كله</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Soft, caramel-rich Medjool dates from Siwa. Hand-graded, never pressed. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">A fridge full of colour makes the healthy choice the easy one. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">أول حاجة بيقدّمها المُضيف. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">كُل قوس قزح كله. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -1517,14 +1517,14 @@
       <c r="C24" s="7">
         <v>46352</v>
       </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Living Well</t>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Box</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pattern card</t>
+          <t xml:space="preserve">Packaging feature</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -1534,27 +1534,27 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rinse herbs just before serving.</t>
+          <t xml:space="preserve">Six herbs. One jar that keeps growing.</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">اغسل الأعشاب قبل التقديم على طول</t>
+          <t xml:space="preserve">الجنينة — ٦ أعشاب وبرطمان بيكبر</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Our herbs arrive washed and dry. For the brightest flavour, give them one more rinse just before you serve. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The Garden box: six herb bunches standing in sleeves, plus a jar of live basil. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">اغسل الأعشاب قبل التقديم على طول. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">الجنينة — ٦ أعشاب وبرطمان بيكبر. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
@@ -1580,14 +1580,14 @@
       <c r="C25" s="7">
         <v>46355</v>
       </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Box</t>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Table</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box feature</t>
+          <t xml:space="preserve">Giant word + produce</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -1597,27 +1597,27 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Herbs, standing in their own sleeves.</t>
+          <t xml:space="preserve">Dates first. Always.</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">أعشاب واقفة كل واحدة في جرابها</t>
+          <t xml:space="preserve">التمر الأول — دايمًا</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Garden box keeps six bunches upright so nothing bruises — plus a jar of live basil. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The host’s first gesture: a small bowl of Medjool dates by the door, before anything else. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">أعشاب واقفة كل واحدة في جرابها. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">التمر الأول — دايمًا. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #سفرة #ضيافة #Hosting #CairoHosting #NewCairo #SheikhZayed</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product on white</t>
+          <t xml:space="preserve">Giant word + produce</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -1660,22 +1660,22 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">A board, in one bunch.</t>
+          <t xml:space="preserve">Red, ripe, and ready.</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">بورد كامل في عنقود واحد</t>
+          <t xml:space="preserve">فراولة — حمرا ومستوية</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plump red grapes from Minya — the quickest way to dress a table. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Winter strawberries are back. Picked at full colour and chilled within hours. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J26" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">بورد كامل في عنقود واحد. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">فراولة — حمرا ومستوية. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -1706,14 +1706,14 @@
       <c r="C27" s="7">
         <v>46357</v>
       </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Living Well</t>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The A Standard</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lifestyle photo</t>
+          <t xml:space="preserve">Split: type over produce</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -1723,27 +1723,27 @@
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Her first strawberry.</t>
+          <t xml:space="preserve">Grade A, only.</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">أول فراولاية</t>
+          <t xml:space="preserve">درجة A بس — مفيش درجة تانية</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Some moments are small and perfect. This was one of them. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Only the first pick of each lot makes it into a Fresh Valley box. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J27" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">أول فراولاية. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">درجة A بس — مفيش درجة تانية. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
@@ -1769,14 +1769,14 @@
       <c r="C28" s="7">
         <v>46358</v>
       </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The A Standard</t>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Living Well</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Framed photo</t>
+          <t xml:space="preserve">Scattered letters</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -1786,27 +1786,27 @@
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Graded where it grows.</t>
+          <t xml:space="preserve">A greener breakfast.</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">بيتفرز مكان ما بيطلع</t>
+          <t xml:space="preserve">فطار أخضر</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Our graders work in the orchard rows, so the best pieces never travel twice. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Avocado, herbs and whatever is in season — breakfast that starts in the garden. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">بيتفرز مكان ما بيطلع. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">فطار أخضر. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr">
@@ -1832,14 +1832,14 @@
       <c r="C29" s="7">
         <v>46359</v>
       </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Table</t>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Box</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Host tip</t>
+          <t xml:space="preserve">Wordmark block</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -1849,27 +1849,27 @@
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">One big bunch beats ten small bowls.</t>
+          <t xml:space="preserve">Three lanes. One salad.</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">عنقود كبير أحسن من عشر أطباق</t>
+          <t xml:space="preserve">سفرة السلطة — ٣ خانات</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A single generous bunch of grapes in the middle of the table makes the whole spread feel abundant. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The Salad Table box: greens, tomatoes and cucumbers in their own lanes, herbs and lemons on the side. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">عنقود كبير أحسن من عشر أطباق. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">سفرة السلطة — ٣ خانات. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #سفرة #ضيافة #Hosting #CairoHosting #NewCairo #SheikhZayed</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split photo</t>
+          <t xml:space="preserve">Four colour tiles</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -1912,22 +1912,22 @@
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Set it from above.</t>
+          <t xml:space="preserve">Four things every host needs.</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">رتّبها من فوق</t>
+          <t xml:space="preserve">٤ حاجات كل مضيف محتاجها</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grapes in the centre, figs and dates around, mint and water glasses at every place. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Grapes, dates, strawberries and mint — the four things that make a tray. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">رتّبها من فوق. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">٤ حاجات كل مضيف محتاجها. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -1958,14 +1958,14 @@
       <c r="C31" s="7">
         <v>46363</v>
       </c>
-      <c r="D31" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Box</t>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Season</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pattern card</t>
+          <t xml:space="preserve">Giant word + produce</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -1975,27 +1975,27 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The lid becomes a poster.</t>
+          <t xml:space="preserve">Autumn’s jewel.</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الغطا يبقى بوستر</t>
+          <t xml:space="preserve">رمان أسيوط</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inside every lid: the Egyptian seasons. Cut along the line and frame it. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Pomegranates from Assiut — heavy, deep red and delivered whole. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الغطا يبقى بوستر. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">رمان أسيوط. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr">
@@ -2021,14 +2021,14 @@
       <c r="C32" s="7">
         <v>46364</v>
       </c>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In Season</t>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The A Standard</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Angle grid</t>
+          <t xml:space="preserve">Type statement</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -2038,27 +2038,27 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mango &amp; stone fruit.</t>
+          <t xml:space="preserve">Nothing added. Nothing hidden.</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">مانجا وفاكهة بنواة</t>
+          <t xml:space="preserve">متغسل — من غير شمع</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ismailia mangoes and Beheira peaches: the taste of an Egyptian summer. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">We wash every piece by hand and never wax it. What you see is the fruit. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J32" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">مانجا وفاكهة بنواة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">متغسل — من غير شمع. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr">
@@ -2084,14 +2084,14 @@
       <c r="C33" s="7">
         <v>46365</v>
       </c>
-      <c r="D33" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The A Standard</t>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Living Well</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type on forest</t>
+          <t xml:space="preserve">Glass pill on green</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -2101,27 +2101,27 @@
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Order by 1 pm. At your door today.</t>
+          <t xml:space="preserve">A bowl of lemons changes the room.</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">اطلب قبل ١ — يوصلك النهارده</t>
+          <t xml:space="preserve">طبق ليمون بيغيّر المكان</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Order before 1 pm and choose a slot today between 4 and 9 pm. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The first thing on the island every morning: a bowl of lemons, delivered the day they’re picked. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">اطلب قبل ١ — يوصلك النهارده. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">طبق ليمون بيغيّر المكان. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr">
@@ -2147,14 +2147,14 @@
       <c r="C34" s="7">
         <v>46366</v>
       </c>
-      <c r="D34" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Living Well</t>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Box</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lifestyle photo</t>
+          <t xml:space="preserve">Packaging feature</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -2164,27 +2164,27 @@
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Slow mornings taste better.</t>
+          <t xml:space="preserve">Arrives as a tray.</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الصبح الهادي طعمه أحلى</t>
+          <t xml:space="preserve">الضيافة — بتوصل صينية</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strawberries, figs and a cup of coffee on the terrace. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The Host box arrives as a serving tray: grapes in the middle, dates, figs, strawberries and mint around it. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الصبح الهادي طعمه أحلى. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">الضيافة — بتوصل صينية. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr">
@@ -2210,14 +2210,14 @@
       <c r="C35" s="7">
         <v>46369</v>
       </c>
-      <c r="D35" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Box</t>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Season</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box feature</t>
+          <t xml:space="preserve">Giant word + produce</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -2227,27 +2227,27 @@
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The week’s market, sorted.</t>
+          <t xml:space="preserve">Summer starts here.</t>
         </is>
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">سوق الأسبوع كله مترتب</t>
+          <t xml:space="preserve">مانجا الإسماعيلية</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Market box: fruit on the left, vegetables on the right — everything the week needs. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Mango season in Ismailia. Picked at the right moment so it is ripe on arrival. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">سوق الأسبوع كله مترتب. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">مانجا الإسماعيلية. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr">
@@ -2273,14 +2273,14 @@
       <c r="C36" s="7">
         <v>46370</v>
       </c>
-      <c r="D36" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The A Standard</t>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Season</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Framed photo</t>
+          <t xml:space="preserve">Scattered letters</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -2290,27 +2290,27 @@
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">From the farm to your gate.</t>
+          <t xml:space="preserve">The one everyone asks for.</t>
         </is>
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">من المزرعة لحد بابك</t>
+          <t xml:space="preserve">مانجا زبدية</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Our riders cover East and West Cairo every afternoon — in insulated bags, so everything arrives as it left. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Zebdia mango — the one every Egyptian table asks for. Back from July to September. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">من المزرعة لحد بابك. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">مانجا زبدية. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr">
@@ -2336,14 +2336,14 @@
       <c r="C37" s="7">
         <v>46371</v>
       </c>
-      <c r="D37" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In Season</t>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The A Standard</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product on white</t>
+          <t xml:space="preserve">Label strips</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -2353,27 +2353,27 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deep red, kept whole.</t>
+          <t xml:space="preserve">Ripened on the vine.</t>
         </is>
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">أحمر غامق — كامل زي ما هو</t>
+          <t xml:space="preserve">طماطم مستوية على عرشها</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Heavy, glossy pomegranates from Assiut. Sold whole, always. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Our tomatoes ripen on the vine and are picked red. They taste like tomatoes again. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">أحمر غامق — كامل زي ما هو. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">طماطم مستوية على عرشها. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split photo</t>
+          <t xml:space="preserve">Split: type over produce</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -2416,22 +2416,22 @@
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">A fridge you want to open.</t>
+          <t xml:space="preserve">Summer in a bowl.</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">تلاجة نفسك تفتحها</t>
+          <t xml:space="preserve">الصيف في طبق</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Herbs in water, berries in glass, vegetables in the crisper — how our customers keep the week fresh. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Peaches, plums and cherries — summer in a bowl. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">تلاجة نفسك تفتحها. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">الصيف في طبق. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
@@ -2462,14 +2462,14 @@
       <c r="C39" s="7">
         <v>46373</v>
       </c>
-      <c r="D39" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Table</t>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Box</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Host tip</t>
+          <t xml:space="preserve">Wordmark block</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -2479,27 +2479,27 @@
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mint in the water, always.</t>
+          <t xml:space="preserve">One box. Six fruits.</t>
         </is>
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">نعناع في المية — دايمًا</t>
+          <t xml:space="preserve">بوكس واحد — ٦ فواكه</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A sprig of fresh mint in every glass of water. Small, and everyone notices. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The Orchard: six fruits at their peak, each in its own well. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J39" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">نعناع في المية — دايمًا. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">بوكس واحد — ٦ فواكه. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #سفرة #ضيافة #Hosting #CairoHosting #NewCairo #SheikhZayed</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lifestyle photo</t>
+          <t xml:space="preserve">Produce crowd + serif</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -2542,22 +2542,22 @@
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Break the fast around one table.</t>
+          <t xml:space="preserve">The table is the point.</t>
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">نفطر على سفرة واحدة</t>
+          <t xml:space="preserve">السفرة هي الحكاية</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dates, figs and grapes on the iftar table — picked and delivered the same day. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Friday lunch. Everything on the table was picked this week. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">نفطر على سفرة واحدة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">السفرة هي الحكاية. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Season card</t>
+          <t xml:space="preserve">Giant word + produce</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -2605,22 +2605,22 @@
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">In season: December</t>
+          <t xml:space="preserve">Green, and proud of it.</t>
         </is>
       </c>
       <c r="H41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">في موسمه: ديسمبر</t>
+          <t xml:space="preserve">بروكلي</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">December’s best: navel oranges, the first strawberries, pears, sweet carrots and lemons. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Tight green broccoli heads, cut the morning they ship. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">في موسمه: ديسمبر. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">بروكلي. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
@@ -2651,14 +2651,14 @@
       <c r="C42" s="7">
         <v>46378</v>
       </c>
-      <c r="D42" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Box</t>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The A Standard</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Framed photo</t>
+          <t xml:space="preserve">Type statement</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -2668,27 +2668,27 @@
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Return the crate. Get 50 EGP off.</t>
+          <t xml:space="preserve">Wrapped in paper.</t>
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">رجّع الصندوق وخد خصم ٥٠</t>
+          <t xml:space="preserve">متلفوف في ورق</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Our wooden crates go round and round. Hand it back on your next delivery and take 50 EGP off. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Every box is kraft, every wrap is paper, and every piece has a second life. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">رجّع الصندوق وخد خصم ٥٠. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">متلفوف في ورق. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
         </is>
       </c>
       <c r="L42" s="6" t="inlineStr">
@@ -2714,14 +2714,14 @@
       <c r="C43" s="7">
         <v>46379</v>
       </c>
-      <c r="D43" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The A Standard</t>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Living Well</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product on white</t>
+          <t xml:space="preserve">Glass pill on green</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
@@ -2731,27 +2731,27 @@
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut to order, still lively.</t>
+          <t xml:space="preserve">Keep it growing.</t>
         </is>
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">بيتقطف حسب الطلب</t>
+          <t xml:space="preserve">خليه يكبر على الشباك</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mint from Qalyubia, cut the morning it ships and bunched by hand. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Our live herbs keep growing on the windowsill. Water them every day. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">بيتقطف حسب الطلب. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">خليه يكبر على الشباك. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
         </is>
       </c>
       <c r="L43" s="6" t="inlineStr">
@@ -2777,14 +2777,14 @@
       <c r="C44" s="7">
         <v>46380</v>
       </c>
-      <c r="D44" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Living Well</t>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Box</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pattern card</t>
+          <t xml:space="preserve">Packaging feature</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -2794,27 +2794,27 @@
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Basil in two weeks.</t>
+          <t xml:space="preserve">Greens, sorted.</t>
         </is>
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ريحان في أسبوعين</t>
+          <t xml:space="preserve">سفرة السلطة</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Soak the seed card, lay it on soil, cover lightly and water daily. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The Salad Table box: three lanes of greens, tomatoes and cucumbers, with herbs and lemons on the side. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ريحان في أسبوعين. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">سفرة السلطة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
         </is>
       </c>
       <c r="L44" s="6" t="inlineStr">
@@ -2840,14 +2840,14 @@
       <c r="C45" s="7">
         <v>46383</v>
       </c>
-      <c r="D45" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Box</t>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Season</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box feature</t>
+          <t xml:space="preserve">Season card</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -2857,27 +2857,27 @@
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The salad course, in three lanes.</t>
+          <t xml:space="preserve">In season: November</t>
         </is>
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">طبق السلطة في ٣ خانات</t>
+          <t xml:space="preserve">في موسمه: نوفمبر</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lettuce and arugula, tomatoes, cucumbers, herbs and lemons — the salad course, sorted. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">November brings the first oranges and strawberries, guava, persimmon, cabbage and carrots. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">طبق السلطة في ٣ خانات. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">في موسمه: نوفمبر. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
         </is>
       </c>
       <c r="L45" s="6" t="inlineStr">
@@ -2903,14 +2903,14 @@
       <c r="C46" s="7">
         <v>46384</v>
       </c>
-      <c r="D46" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Living Well</t>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Table</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lifestyle photo</t>
+          <t xml:space="preserve">Scattered letters</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -2920,27 +2920,27 @@
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lawn, linen, and a basket of fruit.</t>
+          <t xml:space="preserve">Break the fast with something whole.</t>
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">نجيلة، مفرش، وسلة فاكهة</t>
+          <t xml:space="preserve">إفطار على حاجة كاملة</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Weekend picnic in the compound: peaches, apricots, grapes and strawberries. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Dates, pomegranates and fresh juice — iftar starts with something whole. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">نجيلة، مفرش، وسلة فاكهة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">إفطار على حاجة كاملة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #سفرة #ضيافة #Hosting #CairoHosting #NewCairo #SheikhZayed</t>
         </is>
       </c>
       <c r="L46" s="6" t="inlineStr">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type on forest</t>
+          <t xml:space="preserve">Label strips</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
@@ -2983,22 +2983,22 @@
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">No soil. No dust.</t>
+          <t xml:space="preserve">It should snap.</t>
         </is>
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">من غير طين ولا تراب</t>
+          <t xml:space="preserve">الخيار لازم يطرقع</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everything is cleaned and dried before it’s packed — no soil, no dust. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">A good cucumber snaps. Ours are picked young, crisp and thin-skinned. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">من غير طين ولا تراب. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">الخيار لازم يطرقع. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K47" s="5" t="inlineStr">
@@ -3029,14 +3029,14 @@
       <c r="C48" s="7">
         <v>46386</v>
       </c>
-      <c r="D48" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In Season</t>
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Living Well</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Angle grid</t>
+          <t xml:space="preserve">Four colour tiles</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
@@ -3046,27 +3046,27 @@
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Salad staples.</t>
+          <t xml:space="preserve">Colours kids will eat.</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">أساسيات السلطة</t>
+          <t xml:space="preserve">ألوان الولاد هياكلوها</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carrots, vine tomatoes, baladi cucumbers and peppers — the base of every Egyptian salad. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Orange, yellow, green and purple — the easiest way to get vegetables on a child’s plate. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">أساسيات السلطة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">ألوان الولاد هياكلوها. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr">
@@ -3092,14 +3092,14 @@
       <c r="C49" s="7">
         <v>46387</v>
       </c>
-      <c r="D49" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Table</t>
+      <c r="D49" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Box</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split photo</t>
+          <t xml:space="preserve">Wordmark block</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
@@ -3109,27 +3109,27 @@
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fruit is the flowers.</t>
+          <t xml:space="preserve">Herbs, boxed.</t>
         </is>
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الفاكهة هي الورد</t>
+          <t xml:space="preserve">الجنينة — أعشاب في بوكس</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pomegranates, figs and grapes with vine leaves — a centrepiece you can eat. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The Garden box: six herbs standing in sleeves, and a jar of basil that keeps growing. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الفاكهة هي الورد. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">الجنينة — أعشاب في بوكس. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #سفرة #ضيافة #Hosting #CairoHosting #NewCairo #SheikhZayed</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr">
@@ -3155,14 +3155,14 @@
       <c r="C50" s="7">
         <v>46390</v>
       </c>
-      <c r="D50" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In Season</t>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Table</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product on white</t>
+          <t xml:space="preserve">Giant word + produce</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
@@ -3172,27 +3172,27 @@
       </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Honey, in a skin.</t>
+          <t xml:space="preserve">The whole summer.</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">عسل في قشرة</t>
+          <t xml:space="preserve">بطيخ — الصيف كله</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Purple figs from Matrouh. Soft, sweet and whole. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">A whole watermelon on the table is the start of every summer gathering. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">عسل في قشرة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">بطيخ — الصيف كله. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #سفرة #ضيافة #Hosting #CairoHosting #NewCairo #SheikhZayed</t>
         </is>
       </c>
       <c r="L50" s="6" t="inlineStr">
@@ -3218,14 +3218,14 @@
       <c r="C51" s="7">
         <v>46391</v>
       </c>
-      <c r="D51" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Box</t>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Season</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Framed photo</t>
+          <t xml:space="preserve">Scattered letters</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
@@ -3235,27 +3235,27 @@
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The tissue becomes a runner.</t>
+          <t xml:space="preserve">Short season. Don’t miss it.</t>
         </is>
       </c>
       <c r="H51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ورق اللف يبقى رانر</t>
+          <t xml:space="preserve">خرشوف</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unfold the tissue from your box — it’s printed to run down the middle of your table. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Artichoke season is short. Tight, heavy heads, delivered whole. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ورق اللف يبقى رانر. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">خرشوف. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
         </is>
       </c>
       <c r="L51" s="6" t="inlineStr">
@@ -3281,14 +3281,14 @@
       <c r="C52" s="7">
         <v>46392</v>
       </c>
-      <c r="D52" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Living Well</t>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The A Standard</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lifestyle photo</t>
+          <t xml:space="preserve">Type statement</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
@@ -3298,27 +3298,27 @@
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cold grapes, warm afternoon.</t>
+          <t xml:space="preserve">Picked today. Yours today.</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">عنب ساقع وعصرية دافية</t>
+          <t xml:space="preserve">اتقطف النهارده — عندك النهارده</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grapes and cherries by the pool. The simple version of a perfect afternoon. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Same-day delivery across New Cairo, Sheikh Zayed, October, Madinaty and Rehab. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">عنب ساقع وعصرية دافية. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">اتقطف النهارده — عندك النهارده. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
         </is>
       </c>
       <c r="L52" s="6" t="inlineStr">
@@ -3344,14 +3344,14 @@
       <c r="C53" s="7">
         <v>46393</v>
       </c>
-      <c r="D53" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The A Standard</t>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Living Well</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Framed photo</t>
+          <t xml:space="preserve">Produce crowd + serif</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
@@ -3361,27 +3361,27 @@
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Graders, packers, riders.</t>
+          <t xml:space="preserve">Green is a habit.</t>
         </is>
       </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الفرز والتعبئة والتوصيل</t>
+          <t xml:space="preserve">الأخضر عادة</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The people behind every box: graders in the orchard, packers in Obour and riders across Cairo. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Herbs, greens and green fruit — small habits that add up. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الفرز والتعبئة والتوصيل. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">الأخضر عادة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
         </is>
       </c>
       <c r="L53" s="6" t="inlineStr">
@@ -3407,14 +3407,14 @@
       <c r="C54" s="7">
         <v>46394</v>
       </c>
-      <c r="D54" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Table</t>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Box</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Host tip</t>
+          <t xml:space="preserve">Packaging feature</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
@@ -3424,27 +3424,27 @@
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lemons on the table, not in the fridge.</t>
+          <t xml:space="preserve">Carry it to their door.</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الليمون على السفرة مش في التلاجة</t>
+          <t xml:space="preserve">بوكس الهدية — شيله لحد باب البيت</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A bowl of whole lemons brightens a room and keeps them juicier for a few days. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The carry box: a handle on top, a note inside, and a box of whole fruit for someone you love. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الليمون على السفرة مش في التلاجة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">بوكس الهدية — شيله لحد باب البيت. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #سفرة #ضيافة #Hosting #CairoHosting #NewCairo #SheikhZayed</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
         </is>
       </c>
       <c r="L54" s="6" t="inlineStr">
@@ -3470,14 +3470,14 @@
       <c r="C55" s="7">
         <v>46397</v>
       </c>
-      <c r="D55" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Box</t>
+      <c r="D55" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Season</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box feature</t>
+          <t xml:space="preserve">Season card</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
@@ -3487,27 +3487,27 @@
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">One tray, three sizes.</t>
+          <t xml:space="preserve">In season: December</t>
         </is>
       </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">صينية واحدة — ٣ أحجام</t>
+          <t xml:space="preserve">في موسمه: ديسمبر</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every Table box comes in Petite (2–4), Signature (6–8) and Grand (10–12). Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">December: mandarins, oranges, strawberries, broccoli, cabbage and beetroot. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">صينية واحدة — ٣ أحجام. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">في موسمه: ديسمبر. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
         </is>
       </c>
       <c r="L55" s="6" t="inlineStr">
@@ -3533,14 +3533,14 @@
       <c r="C56" s="7">
         <v>46398</v>
       </c>
-      <c r="D56" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In Season</t>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Table</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Season card</t>
+          <t xml:space="preserve">Split: type over produce</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
@@ -3550,27 +3550,27 @@
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">In season: July</t>
+          <t xml:space="preserve">Winter tastes like this.</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">في موسمه: يوليو</t>
+          <t xml:space="preserve">الشتا طعمه كده</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">High summer: mango season, grapes, figs and peaches. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Mandarins, pomegranates and dates — winter on the table. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">في موسمه: يوليو. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">الشتا طعمه كده. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #EgyptianProduce #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #سفرة #ضيافة #Hosting #CairoHosting #NewCairo #SheikhZayed</t>
         </is>
       </c>
       <c r="L56" s="6" t="inlineStr">
@@ -3596,14 +3596,14 @@
       <c r="C57" s="7">
         <v>46399</v>
       </c>
-      <c r="D57" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Living Well</t>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The A Standard</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split photo</t>
+          <t xml:space="preserve">Label strips</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
@@ -3613,27 +3613,27 @@
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">A basket full of sun.</t>
+          <t xml:space="preserve">Grown for colour.</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">سلة مليانة شمس</t>
+          <t xml:space="preserve">فلفل النوبارية</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Picked whole, with their leaves. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Red, yellow and green peppers from Nubaria — thick walls, glossy skin. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">سلة مليانة شمس. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">فلفل النوبارية. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
         </is>
       </c>
       <c r="L57" s="6" t="inlineStr">
@@ -3659,14 +3659,14 @@
       <c r="C58" s="7">
         <v>46400</v>
       </c>
-      <c r="D58" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The A Standard</t>
+      <c r="D58" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Living Well</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type on forest</t>
+          <t xml:space="preserve">Glass pill on green</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
@@ -3676,27 +3676,27 @@
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Picked whole. Kept whole.</t>
+          <t xml:space="preserve">Lunchbox, sorted.</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">بيتقطف كامل — ويوصل كامل</t>
+          <t xml:space="preserve">شنطة المدرسة متظبطة</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">We sell produce whole — never cut, never opened. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">A crisp green apple in every lunchbox, washed and paper-wrapped. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">بيتقطف كامل — ويوصل كامل. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">شنطة المدرسة متظبطة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
         </is>
       </c>
       <c r="L58" s="6" t="inlineStr">
@@ -3722,14 +3722,14 @@
       <c r="C59" s="7">
         <v>46401</v>
       </c>
-      <c r="D59" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Table</t>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Box</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lifestyle photo</t>
+          <t xml:space="preserve">Packaging feature</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
@@ -3739,27 +3739,27 @@
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stay a little longer.</t>
+          <t xml:space="preserve">Five boxes. Three sizes.</t>
         </is>
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">خليك شوية كمان</t>
+          <t xml:space="preserve">٥ بوكسات — ٣ أحجام</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">String lights, olive trees and a table full of whole fruit and greens. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The Orchard, the Market, the Garden, the Salad Table and the Host — Petite, Signature or Grand. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">خليك شوية كمان. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">٥ بوكسات — ٣ أحجام. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #سفرة #ضيافة #Hosting #CairoHosting #NewCairo #SheikhZayed</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
         </is>
       </c>
       <c r="L59" s="6" t="inlineStr">
@@ -3785,14 +3785,14 @@
       <c r="C60" s="7">
         <v>46404</v>
       </c>
-      <c r="D60" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Box</t>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Table</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Framed photo</t>
+          <t xml:space="preserve">Four colour tiles</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
@@ -3802,27 +3802,27 @@
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">From our hands to yours.</t>
+          <t xml:space="preserve">Never the same twice.</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">من إيدنا لإيدك</t>
+          <t xml:space="preserve">طبق الفاكهة عمره ما يتكرر</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every Host box is handed over at the door — never left on a step. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">The fruit bowl changes every week because the season does. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">من إيدنا لإيدك. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">طبق الفاكهة عمره ما يتكرر. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #سفرة #ضيافة #Hosting #CairoHosting #NewCairo #SheikhZayed</t>
         </is>
       </c>
       <c r="L60" s="6" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product on white</t>
+          <t xml:space="preserve">Giant word + produce</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
@@ -3865,22 +3865,22 @@
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Worth the wait.</t>
+          <t xml:space="preserve">You’ll smell it at the door.</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">تستاهل الاستنا</t>
+          <t xml:space="preserve">جوافة — ريحتها قبلها</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ismailia mangoes, golden and blushing red. The fruit Egypt waits all year for. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Guava season. You’ll smell the box before you open it. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">تستاهل الاستنا. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">جوافة — ريحتها قبلها. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K61" s="5" t="inlineStr">
@@ -3911,14 +3911,14 @@
       <c r="C62" s="7">
         <v>46406</v>
       </c>
-      <c r="D62" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Living Well</t>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The A Standard</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lifestyle photo</t>
+          <t xml:space="preserve">Type statement</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
@@ -3928,27 +3928,27 @@
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recipes start here.</t>
+          <t xml:space="preserve">Not right? Not your problem.</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الوصفات بتبدأ من هنا</t>
+          <t xml:space="preserve">مش مظبوط؟ مش مشكلتك</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sorting herbs with teta — where every family recipe starts. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">If anything isn’t right, it isn’t your problem. Send a photo and we fix it. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">الوصفات بتبدأ من هنا. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">مش مظبوط؟ مش مشكلتك. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
         </is>
       </c>
       <c r="L62" s="6" t="inlineStr">
@@ -3974,14 +3974,14 @@
       <c r="C63" s="7">
         <v>46407</v>
       </c>
-      <c r="D63" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The A Standard</t>
+      <c r="D63" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Living Well</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pattern card</t>
+          <t xml:space="preserve">Scattered letters</t>
         </is>
       </c>
       <c r="F63" s="6" t="inlineStr">
@@ -3991,27 +3991,27 @@
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not right? We replace it.</t>
+          <t xml:space="preserve">More plants, every day.</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">مش مظبوط؟ بنبدّله</t>
+          <t xml:space="preserve">خضار أكتر كل يوم</t>
         </is>
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Send a photo on WhatsApp within 24 hours — we replace it or refund it. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Crisp romaine, cut this morning. The easiest way to eat more plants. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">مش مظبوط؟ بنبدّله. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">خضار أكتر كل يوم. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد #Cairo</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #SlowMornings #HomeInCairo #كمباوند #Wellness</t>
         </is>
       </c>
       <c r="L63" s="6" t="inlineStr">
@@ -4037,14 +4037,14 @@
       <c r="C64" s="7">
         <v>46408</v>
       </c>
-      <c r="D64" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Table</t>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Box</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type on forest</t>
+          <t xml:space="preserve">Wordmark block</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
@@ -4054,27 +4054,27 @@
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOST10 10% off your first table.</t>
+          <t xml:space="preserve">Picked this morning. At your table today.</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">خصم ١٠٪ على أول سفرة</t>
+          <t xml:space="preserve">اتقطف الصبح — على سفرتك النهارده</t>
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use HOST10 for 10% off your first order. Order by 1 pm — at your door today.</t>
+          <t xml:space="preserve">Order on the site or on WhatsApp before noon for same-day delivery. Order by 1 pm — at your door today.</t>
         </is>
       </c>
       <c r="J64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">خصم ١٠٪ على أول سفرة. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
+          <t xml:space="preserve">اتقطف الصبح — على سفرتك النهارده. اطلب قبل ١ الضهر — يوصلك النهارده. الرابط في البايو.</t>
         </is>
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #سفرة #ضيافة #Hosting #CairoHosting #NewCairo #SheikhZayed</t>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting #هدايا</t>
         </is>
       </c>
       <c r="L64" s="6" t="inlineStr">
@@ -4205,7 +4205,7 @@
         </is>
       </c>
       <c r="G5" s="6">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is at its best right now — month cards, hero fruit, angle grids. Always whole, never cut.</t>
+          <t xml:space="preserve">What is at its best right now — month cards, giant-word hero fruit, colour tiles. Always whole, never cut.</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -4265,7 +4265,7 @@
         </is>
       </c>
       <c r="G7" s="6">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
@@ -4286,7 +4286,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mornings, kids, herbs on the windowsill, the organised fridge. Villa and compound life in natural light.</t>
+          <t xml:space="preserve">Mornings, kids, herbs on the windowsill, the organised fridge. Told through produce and type only — no people.</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -4325,7 +4325,7 @@
         </is>
       </c>
       <c r="G9" s="6">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">

</xml_diff>